<commit_message>
Add Power Supply BOM: Zener gate protection + LM2576 regulators
- เพิ่ม 1N4746A (18V Zener) ป้องกัน gate MOSFET ×6 ตัว
- เพิ่ม LM2576HVT-12 + อุปกรณ์ประกอบ (48V→12V สำหรับ Gate Driver)
- เพิ่ม LM2576T-5.0 + อุปกรณ์ประกอบ (12V→5V สำหรับ ESP32)
- อัปเดต BOM รวม 20 รายการ พร้อม SUM formula

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/claude_MOSFET_GateDriver_Selection_48V_500W.xlsx
+++ b/claude_MOSFET_GateDriver_Selection_48V_500W.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Design Parameters" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="MOSFET Selection" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Gate Driver Selection" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="BOM (Recommended)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Gate Drive Circuit" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Parameters" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MOSFET Selection" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate Driver Selection" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM (Recommended)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate Drive Circuit" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -70,7 +70,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -117,8 +117,26 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+        <bgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -198,11 +216,55 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="002E75B6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="002E75B6"/>
+      </right>
+      <top style="medium">
+        <color rgb="002E75B6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="002E75B6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002E75B6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="002E75B6"/>
+      </right>
+      <top style="medium">
+        <color rgb="002E75B6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002E75B6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -296,6 +358,26 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -679,6 +761,11 @@
           <t>🔧  Inverter Design Parameters  |  48 V / 500 W Motor Drive</t>
         </is>
       </c>
+      <c r="B1" s="34" t="n"/>
+      <c r="C1" s="34" t="n"/>
+      <c r="D1" s="34" t="n"/>
+      <c r="E1" s="34" t="n"/>
+      <c r="F1" s="35" t="n"/>
     </row>
     <row r="2" ht="6" customHeight="1"/>
     <row r="3">
@@ -1046,6 +1133,18 @@
           <t>⚡  MOSFET Selection  |  48 V / 500 W Motor Inverter  |  หาซื้อได้ใน Shopee ไทย</t>
         </is>
       </c>
+      <c r="B1" s="34" t="n"/>
+      <c r="C1" s="34" t="n"/>
+      <c r="D1" s="34" t="n"/>
+      <c r="E1" s="34" t="n"/>
+      <c r="F1" s="34" t="n"/>
+      <c r="G1" s="34" t="n"/>
+      <c r="H1" s="34" t="n"/>
+      <c r="I1" s="34" t="n"/>
+      <c r="J1" s="34" t="n"/>
+      <c r="K1" s="34" t="n"/>
+      <c r="L1" s="34" t="n"/>
+      <c r="M1" s="35" t="n"/>
     </row>
     <row r="2" ht="6" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
@@ -1680,6 +1779,17 @@
           <t>🔌  Gate Driver Selection  |  48 V Inverter  |  หาซื้อได้ใน Shopee ไทย</t>
         </is>
       </c>
+      <c r="B1" s="34" t="n"/>
+      <c r="C1" s="34" t="n"/>
+      <c r="D1" s="34" t="n"/>
+      <c r="E1" s="34" t="n"/>
+      <c r="F1" s="34" t="n"/>
+      <c r="G1" s="34" t="n"/>
+      <c r="H1" s="34" t="n"/>
+      <c r="I1" s="34" t="n"/>
+      <c r="J1" s="34" t="n"/>
+      <c r="K1" s="34" t="n"/>
+      <c r="L1" s="35" t="n"/>
     </row>
     <row r="2" ht="6" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
@@ -2213,7 +2323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2232,6 +2342,13 @@
           <t>📋  BOM – ชุดแนะนำสำหรับ Inverter 3-Phase 48V / 500W</t>
         </is>
       </c>
+      <c r="B1" s="34" t="n"/>
+      <c r="C1" s="34" t="n"/>
+      <c r="D1" s="34" t="n"/>
+      <c r="E1" s="34" t="n"/>
+      <c r="F1" s="34" t="n"/>
+      <c r="G1" s="34" t="n"/>
+      <c r="H1" s="35" t="n"/>
     </row>
     <row r="2" ht="6" customHeight="1"/>
     <row r="3" ht="30" customHeight="1">
@@ -2591,22 +2708,426 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="26" t="inlineStr">
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" s="41" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="41" t="inlineStr">
+        <is>
+          <t>Gate Protection Zener</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>1N4746A (18V 1W)</t>
+        </is>
+      </c>
+      <c r="D13" s="41" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" s="41" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" s="41">
+        <f>D13*E13</f>
+        <v/>
+      </c>
+      <c r="G13" s="37" t="inlineStr">
+        <is>
+          <t>Clamp Vgs ≤ 18V ต่อ Gate–Source ทุก MOSFET DO-41</t>
+        </is>
+      </c>
+      <c r="H13" s="41" t="inlineStr">
+        <is>
+          <t>1N4746A zener 18V</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="38" t="inlineStr">
+        <is>
+          <t>⚡  Power Supply — Gate Driver VCC (48V → 12V)  |  LM2576HVT-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
+      <c r="A15" s="39" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="39" t="inlineStr">
+        <is>
+          <t>Buck Regulator 48V→12V</t>
+        </is>
+      </c>
+      <c r="C15" s="39" t="inlineStr">
+        <is>
+          <t>LM2576HVT-12</t>
+        </is>
+      </c>
+      <c r="D15" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="39" t="n">
+        <v>60</v>
+      </c>
+      <c r="F15" s="39">
+        <f>D15*E15</f>
+        <v/>
+      </c>
+      <c r="G15" s="40" t="inlineStr">
+        <is>
+          <t>3A Step-Down ทน 60V สำหรับ Gate Driver VCC</t>
+        </is>
+      </c>
+      <c r="H15" s="39" t="inlineStr">
+        <is>
+          <t>LM2576HVT-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="39" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="39" t="inlineStr">
+        <is>
+          <t>Inductor L1 (48V→12V)</t>
+        </is>
+      </c>
+      <c r="C16" s="39" t="inlineStr">
+        <is>
+          <t>100µH 3A Ferrite</t>
+        </is>
+      </c>
+      <c r="D16" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="39" t="n">
+        <v>35</v>
+      </c>
+      <c r="F16" s="39">
+        <f>D16*E16</f>
+        <v/>
+      </c>
+      <c r="G16" s="40" t="inlineStr">
+        <is>
+          <t>อิ่มตัว ≥ 3A แกน ferrite</t>
+        </is>
+      </c>
+      <c r="H16" s="39" t="inlineStr">
+        <is>
+          <t>inductor 100uH 3A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="39" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="39" t="inlineStr">
+        <is>
+          <t>Catch Diode D1 (48V→12V)</t>
+        </is>
+      </c>
+      <c r="C17" s="39" t="inlineStr">
+        <is>
+          <t>1N5822 Schottky 3A</t>
+        </is>
+      </c>
+      <c r="D17" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="F17" s="39">
+        <f>D17*E17</f>
+        <v/>
+      </c>
+      <c r="G17" s="40" t="inlineStr">
+        <is>
+          <t>Schottky 3A/40V fast recovery</t>
+        </is>
+      </c>
+      <c r="H17" s="39" t="inlineStr">
+        <is>
+          <t>1N5822 Schottky</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="39" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="39" t="inlineStr">
+        <is>
+          <t>Input Cap Cin1 (48V→12V)</t>
+        </is>
+      </c>
+      <c r="C18" s="39" t="inlineStr">
+        <is>
+          <t>100µF 63V Electrolytic</t>
+        </is>
+      </c>
+      <c r="D18" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="39" t="n">
+        <v>12</v>
+      </c>
+      <c r="F18" s="39">
+        <f>D18*E18</f>
+        <v/>
+      </c>
+      <c r="G18" s="40" t="inlineStr">
+        <is>
+          <t>ทนแรงดัน ≥ 63V ต่อขา Vin LM2576HVT</t>
+        </is>
+      </c>
+      <c r="H18" s="39" t="inlineStr">
+        <is>
+          <t>capacitor 100uF 63V</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="39" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="39" t="inlineStr">
+        <is>
+          <t>Output Cap Cout1 (48V→12V)</t>
+        </is>
+      </c>
+      <c r="C19" s="39" t="inlineStr">
+        <is>
+          <t>100µF 25V Electrolytic</t>
+        </is>
+      </c>
+      <c r="D19" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="F19" s="39">
+        <f>D19*E19</f>
+        <v/>
+      </c>
+      <c r="G19" s="40" t="inlineStr">
+        <is>
+          <t>Output filter ต่อขา Output</t>
+        </is>
+      </c>
+      <c r="H19" s="39" t="inlineStr">
+        <is>
+          <t>capacitor 100uF 25V</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="38" t="inlineStr">
+        <is>
+          <t>⚡  Power Supply — MCU/ESP32 Supply (12V → 5V)  |  LM2576T-5.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="39" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="39" t="inlineStr">
+        <is>
+          <t>Buck Regulator 12V→5V</t>
+        </is>
+      </c>
+      <c r="C21" s="39" t="inlineStr">
+        <is>
+          <t>LM2576T-5.0</t>
+        </is>
+      </c>
+      <c r="D21" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="39" t="n">
+        <v>40</v>
+      </c>
+      <c r="F21" s="39">
+        <f>D21*E21</f>
+        <v/>
+      </c>
+      <c r="G21" s="40" t="inlineStr">
+        <is>
+          <t>3A Step-Down Fixed 5V สำหรับ ESP32</t>
+        </is>
+      </c>
+      <c r="H21" s="39" t="inlineStr">
+        <is>
+          <t>LM2576T-5.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="39" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" s="39" t="inlineStr">
+        <is>
+          <t>Inductor L2 (12V→5V)</t>
+        </is>
+      </c>
+      <c r="C22" s="39" t="inlineStr">
+        <is>
+          <t>100µH 3A Ferrite</t>
+        </is>
+      </c>
+      <c r="D22" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="39" t="n">
+        <v>35</v>
+      </c>
+      <c r="F22" s="39">
+        <f>D22*E22</f>
+        <v/>
+      </c>
+      <c r="G22" s="40" t="inlineStr">
+        <is>
+          <t>ใช้เบอร์เดียวกับ L1 ได้เลย</t>
+        </is>
+      </c>
+      <c r="H22" s="39" t="inlineStr">
+        <is>
+          <t>inductor 100uH 3A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="39" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" s="39" t="inlineStr">
+        <is>
+          <t>Catch Diode D2 (12V→5V)</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="inlineStr">
+        <is>
+          <t>1N5822 Schottky 3A</t>
+        </is>
+      </c>
+      <c r="D23" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="F23" s="39">
+        <f>D23*E23</f>
+        <v/>
+      </c>
+      <c r="G23" s="40" t="inlineStr">
+        <is>
+          <t>Schottky 3A/40V เหมือน D1</t>
+        </is>
+      </c>
+      <c r="H23" s="39" t="inlineStr">
+        <is>
+          <t>1N5822 Schottky</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" s="39" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" s="39" t="inlineStr">
+        <is>
+          <t>Input Cap Cin2 (12V→5V)</t>
+        </is>
+      </c>
+      <c r="C24" s="39" t="inlineStr">
+        <is>
+          <t>100µF 25V Electrolytic</t>
+        </is>
+      </c>
+      <c r="D24" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="F24" s="39">
+        <f>D24*E24</f>
+        <v/>
+      </c>
+      <c r="G24" s="40" t="inlineStr">
+        <is>
+          <t>ต่อขา Vin LM2576T-5.0</t>
+        </is>
+      </c>
+      <c r="H24" s="39" t="inlineStr">
+        <is>
+          <t>capacitor 100uF 25V</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1">
+      <c r="A25" s="39" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" s="39" t="inlineStr">
+        <is>
+          <t>Output Cap Cout2 (12V→5V)</t>
+        </is>
+      </c>
+      <c r="C25" s="39" t="inlineStr">
+        <is>
+          <t>100µF 10V Electrolytic</t>
+        </is>
+      </c>
+      <c r="D25" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="F25" s="39">
+        <f>D25*E25</f>
+        <v/>
+      </c>
+      <c r="G25" s="40" t="inlineStr">
+        <is>
+          <t>Output filter สำหรับ ESP32 supply</t>
+        </is>
+      </c>
+      <c r="H25" s="39" t="inlineStr">
+        <is>
+          <t>capacitor 100uF 10V</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="26" t="inlineStr">
         <is>
           <t>ประมาณการรวม (฿)</t>
         </is>
       </c>
-      <c r="F13" s="27">
-        <f>SUM(F4:F12)</f>
+      <c r="B26" s="30" t="n"/>
+      <c r="C26" s="30" t="n"/>
+      <c r="D26" s="30" t="n"/>
+      <c r="E26" s="31" t="n"/>
+      <c r="F26" s="27">
+        <f>SUM(F4:F25)</f>
         <v/>
       </c>
-      <c r="G13" s="28" t="inlineStr"/>
-      <c r="H13" s="28" t="inlineStr"/>
+      <c r="G26" s="28" t="inlineStr"/>
+      <c r="H26" s="28" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A13:E13"/>
+  <mergeCells count="3">
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2634,6 +3155,9 @@
           <t>📐  Gate Drive Circuit – คำอธิบายวงจรและการต่อ (IR2110 / EG3013)</t>
         </is>
       </c>
+      <c r="B1" s="34" t="n"/>
+      <c r="C1" s="34" t="n"/>
+      <c r="D1" s="35" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="29" t="inlineStr"/>

</xml_diff>